<commit_message>
Updated Chapter 3 Design 3.1-3.5
</commit_message>
<xml_diff>
--- a/assets/submission checklist.xlsx
+++ b/assets/submission checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cowse\aes-thesis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B32630-591A-43D2-ABFB-C0406E86CA71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2892CCC1-9C97-4040-B233-59120219242C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="48">
   <si>
     <t>Name</t>
   </si>
@@ -153,9 +153,6 @@
     <t>Daria</t>
   </si>
   <si>
-    <t>Scion</t>
-  </si>
-  <si>
     <t>Shanella</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>Bryce</t>
+  </si>
+  <si>
+    <t>Darnell</t>
   </si>
 </sst>
 </file>
@@ -585,7 +585,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -613,7 +613,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -623,7 +623,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
@@ -637,7 +637,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -651,33 +651,36 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
@@ -691,7 +694,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B19" t="s">
         <v>15</v>
@@ -705,32 +708,32 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="B20" t="s">
         <v>15</v>
       </c>
       <c r="C20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
         <v>15</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
         <v>15</v>
@@ -744,50 +747,50 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>34</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
         <v>15</v>
@@ -801,7 +804,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>15</v>
@@ -815,7 +818,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B30" t="s">
         <v>15</v>
@@ -829,18 +832,21 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
         <v>15</v>
       </c>
       <c r="C31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="B32" t="s">
         <v>15</v>
@@ -854,28 +860,37 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34" t="s">
-        <v>15</v>
-      </c>
-      <c r="C34" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -899,8 +914,11 @@
       <c r="C38" t="s">
         <v>15</v>
       </c>
+      <c r="D38" t="s">
+        <v>15</v>
+      </c>
       <c r="G38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -927,6 +945,9 @@
         <v>15</v>
       </c>
       <c r="C41" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Chapter 5 Evaluation, completed input component development
</commit_message>
<xml_diff>
--- a/assets/submission checklist.xlsx
+++ b/assets/submission checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cowse\aes-thesis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2892CCC1-9C97-4040-B233-59120219242C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F17DB9F-5071-48D6-8E5C-EB8BDAAF9B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="48">
   <si>
     <t>Name</t>
   </si>
@@ -558,6 +558,9 @@
       <c r="C4" t="s">
         <v>15</v>
       </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -887,6 +890,9 @@
       <c r="C35" t="s">
         <v>15</v>
       </c>
+      <c r="D35" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
@@ -901,6 +907,9 @@
         <v>15</v>
       </c>
       <c r="C37" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>